<commit_message>
fix: apply review fixes and package 1.6.1
</commit_message>
<xml_diff>
--- a/主线版本对应源地址.xlsx
+++ b/主线版本对应源地址.xlsx
@@ -23824,7 +23824,7 @@
     <hyperlink ref="C66" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2 main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000C main&#10;deb https://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all"/>
     <hyperlink ref="C67" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL  10.1-kirin9000C-2403-feature-bugfix-limit main universe restricted multiverse &#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-kirin9000C-2403-feature main &#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-wayland-2403-updates main universe restricted multiverse&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb http://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all&#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-wayland-2403-updates&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kirin9000C-2403-feature-bugfix-limit &#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kirin9000C-2403-feature &#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: ori"/>
     <hyperlink ref="C68" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL  10.1-kirin9000C-2403-feature-bugfix-limit main universe restricted multiverse &#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-kirin9000C-b-2403-feature main&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-wayland-2403-updates main universe restricted multiverse&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb http://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all&#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-wayland-2403-updates&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kirin9000C-2403-feature-bugfix-limit &#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kirin9000C-b-2403-feature&#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: o"/>
-    <hyperlink ref="C69" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000C-pre-bugfix-limit main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2 main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000C-pre main&#10;deb https://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all  &#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000C-pre&#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a= 10.1-2403-wayland-update2-kirin9000C-pre-bu"/>
+    <hyperlink ref="C69" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000C-pre-bugfix-limit main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2 main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000C-pre main&#10;deb https://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all  &#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000C-pre&#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000C-pre-bu"/>
     <hyperlink ref="C70" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000X-bugfix-limit main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2 main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000X main&#10;deb https://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all&#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000X &#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000X-bugfix-limit&#10;Pin-Pri"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24987,7 +24987,7 @@
     <hyperlink ref="B139" r:id="rId1" display="deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-kylin  main restricted universe multiverse&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-kylin-2503-wayland main universe restricted multiverse&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2503-wayland-bugfix-limit main universe restricted multiverse&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-kylin-2503-wayland-kirin9000C main&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-kylin-2503-wayland-kirin9000C-bugfix main universe restricted multiverse&#10;deb http://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all&#10;&#10;修改/etc/apt/preferences.d/kylin.pref 文件&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin-2503-wayland&#10;Pin-Priority: 600&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2503-wayland-bugfix-limit&#10;Pin-Priority: 600&#10;Package: *&#10;Pin: origin &quot;arch"/>
     <hyperlink ref="B140" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL  10.1-kirin9000C-2403-feature-bugfix-limit main universe restricted multiverse &#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-kirin9000C-2403-feature main &#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-wayland-2403-updates main universe restricted multiverse&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb http://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all&#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-wayland-2403-updates&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kirin9000C-2403-feature-bugfix-limit &#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kirin9000C-2403-feature &#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: ori"/>
     <hyperlink ref="B141" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL  10.1-kirin9000C-2403-feature-bugfix-limit main universe restricted multiverse &#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-kirin9000C-b-2403-feature main&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-wayland-2403-updates main universe restricted multiverse&#10;deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb http://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all&#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-wayland-2403-updates&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kirin9000C-2403-feature-bugfix-limit &#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kirin9000C-b-2403-feature&#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: o"/>
-    <hyperlink ref="B142" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000C-pre-bugfix-limit main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2 main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000C-pre main&#10;deb https://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all  &#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000C-pre&#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a= 10.1-2403-wayland-update2-kirin9000C-pre-bu"/>
+    <hyperlink ref="B142" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000C-pre-bugfix-limit main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2 main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000C-pre main&#10;deb https://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all  &#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000C-pre&#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000C-pre-bu"/>
     <hyperlink ref="B143" r:id="rId3" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000X-bugfix-limit main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2 main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-2403-wayland-update2-kirin9000X main&#10;deb https://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all&#10;优先级设置【/etc/apt/preferences.d/kylin.pref文件】&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-kylin&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2&#10;Pin-Priority: 500&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000X &#10;Pin-Priority: 600&#10;&#10;Package: *&#10;Pin: origin &quot;archive.kylinos.cn&quot;&#10;Pin: release a=10.1-2403-wayland-update2-kirin9000X-bugfix-limit&#10;Pin-Pri"/>
     <hyperlink ref="B144" r:id="rId1" display="deb http://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-pw main restricted universe multiverse"/>
     <hyperlink ref="B145" r:id="rId4" display="deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1 main restricted universe multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-wayland-2403-updates main universe restricted multiverse&#10;deb https://archive.kylinos.cn/kylin/KYLIN-ALL 10.1-kirin9000C-2403-feature main&#10;deb https://archive2.kylinos.cn/deb/kylin/production/PART-10_1-kirin9a0/custom/partner/10_1-kirin9a0 default all"/>

</xml_diff>